<commit_message>
[ROS-PS-v4.2.0] Correct reference links
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ROS-PS/v4.2.0/Form-ROS-PS-v4.2.0.xlsx
+++ b/form_reporting_templates/ROS-PS/v4.2.0/Form-ROS-PS-v4.2.0.xlsx
@@ -6434,7 +6434,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E1" r:id="rId1" location="samplingMethodsForSamplingCollection" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
+    <hyperlink ref="E1" r:id="rId1" location="samplingMethodsForSamplingCollections" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
     <hyperlink ref="O1" r:id="rId2" location="sex" xr:uid="{00000000-0004-0000-0900-000001000000}"/>
     <hyperlink ref="F2" r:id="rIdV420_F2" xr:uid="{00000000-0004-0000-0900-000002000000}" location="allMeasurements"/>
     <hyperlink ref="H2" r:id="rId4" location="lengthMeasurementTools" xr:uid="{00000000-0004-0000-0900-000003000000}"/>
@@ -6443,7 +6443,7 @@
     <hyperlink ref="L2" r:id="rId7" location="fishProcessingTypes" xr:uid="{00000000-0004-0000-0900-000006000000}"/>
     <hyperlink ref="N2" r:id="rId8" location="weightMeasurementTools" xr:uid="{00000000-0004-0000-0900-000007000000}"/>
     <hyperlink ref="Q2" r:id="rIdV420_S2" xr:uid="{00000000-0004-0000-0900-000008000000}" location="maturityStages"/>
-    <hyperlink ref="R2" r:id="rId10" location="samplingMethodsForSamplingCollection" xr:uid="{00000000-0004-0000-0900-000009000000}"/>
+    <hyperlink ref="R2" r:id="rId10" location="biologicalMaterials" xr:uid="{00000000-0004-0000-0900-000009000000}"/>
     <hyperlink ref="S2" r:id="rId11" location="fishStorageTypes" xr:uid="{00000000-0004-0000-0900-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -44083,7 +44083,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D1" r:id="rIdV420_D1" xr:uid="{00000000-0004-0000-0700-000000000000}" location="speciesCetaceans"/>
+    <hyperlink ref="D1" r:id="rIdV420_D1" xr:uid="{00000000-0004-0000-0700-000000000000}" location="cetaceanSpecies"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -46781,7 +46781,7 @@
   <hyperlinks>
     <hyperlink ref="D1" r:id="rIdSpecies420_1" xr:uid="{00000000-0004-0000-0800-000000000000}" location="allSpecies"/>
     <hyperlink ref="G1" r:id="rId2" location="samplingMethodsForCatchEstimation" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
-    <hyperlink ref="E2" r:id="rId3" location="typesOfFate" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
+    <hyperlink ref="E2" r:id="rId3" location="fateTypes" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
     <hyperlink ref="F2" r:id="rId4" location="fates" xr:uid="{00000000-0004-0000-0800-000003000000}"/>
     <hyperlink ref="I2" r:id="rId5" location="fishProcessingTypes" xr:uid="{00000000-0004-0000-0800-000004000000}"/>
     <hyperlink ref="K2" r:id="rIdV420_K2" xr:uid="{00000000-0004-0000-0800-000005000000}" location="weightMeasurementTools"/>

</xml_diff>

<commit_message>
[ROS-PS-v4.2.0] Correct FAD design and sample preservation links
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ROS-PS/v4.2.0/Form-ROS-PS-v4.2.0.xlsx
+++ b/form_reporting_templates/ROS-PS/v4.2.0/Form-ROS-PS-v4.2.0.xlsx
@@ -6444,7 +6444,7 @@
     <hyperlink ref="N2" r:id="rId8" location="weightMeasurementTools" xr:uid="{00000000-0004-0000-0900-000007000000}"/>
     <hyperlink ref="Q2" r:id="rIdV420_S2" xr:uid="{00000000-0004-0000-0900-000008000000}" location="maturityStages"/>
     <hyperlink ref="R2" r:id="rId10" location="biologicalMaterials" xr:uid="{00000000-0004-0000-0900-000009000000}"/>
-    <hyperlink ref="S2" r:id="rId11" location="fishStorageTypes" xr:uid="{00000000-0004-0000-0900-00000A000000}"/>
+    <hyperlink ref="S2" r:id="rId11" location="samplePreservationMethods" xr:uid="{00000000-0004-0000-0900-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -42432,8 +42432,8 @@
     <hyperlink ref="G3" r:id="rId4" location="schoolSightingCues" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
     <hyperlink ref="H3" r:id="rId5" location="schoolSightingCues" xr:uid="{00000000-0004-0000-0600-000004000000}"/>
     <hyperlink ref="I3" r:id="rId6" location="schoolSightingCues" xr:uid="{00000000-0004-0000-0600-000005000000}"/>
-    <hyperlink ref="U3" r:id="rId7" location="FADraftDesigns" xr:uid="{00000000-0004-0000-0600-000006000000}"/>
-    <hyperlink ref="V3" r:id="rId8" location="FADtailDesigns" xr:uid="{00000000-0004-0000-0600-000007000000}"/>
+    <hyperlink ref="U3" r:id="rId7" location="fadRaftDesigns" xr:uid="{00000000-0004-0000-0600-000006000000}"/>
+    <hyperlink ref="V3" r:id="rId8" location="fadTailDesigns" xr:uid="{00000000-0004-0000-0600-000007000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>